<commit_message>
chore: presentation pages cleaned after sensitivity audit
- internal ideas file and preview removed from plan folder
- seller names removed from revenue CSV
- media moved into presentation folder, no links to /invest/
- css comments stripped, model labels and notes neutralized
- internal links removed from kuda and vyruchka

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model-v7/maison-financial-model.xlsx
+++ b/model-v7/maison-financial-model.xlsx
@@ -7073,7 +7073,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">        События и маркеты: грузчики, диджей, расходники</t>
+          <t xml:space="preserve">        События и маркеты: грузчики, музыка, расходники</t>
         </is>
       </c>
       <c r="B43" s="17" t="n">
@@ -8643,7 +8643,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Подписки: сайт Shopify, домен, GPT, Claude, музыка</t>
+          <t xml:space="preserve">        Подписки и сервисы: сайт, домен, музыка, программы</t>
         </is>
       </c>
       <c r="B53" s="17" t="n">
@@ -21070,7 +21070,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">        События и маркеты: грузчики, диджей, расходники</t>
+          <t xml:space="preserve">        События и маркеты: грузчики, музыка, расходники</t>
         </is>
       </c>
       <c r="B43" s="17" t="n">
@@ -22640,7 +22640,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Подписки: сайт Shopify, домен, GPT, Claude, музыка</t>
+          <t xml:space="preserve">        Подписки и сервисы: сайт, домен, музыка, программы</t>
         </is>
       </c>
       <c r="B53" s="17" t="n">
@@ -35067,7 +35067,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">        События и маркеты: грузчики, диджей, расходники</t>
+          <t xml:space="preserve">        События и маркеты: грузчики, музыка, расходники</t>
         </is>
       </c>
       <c r="B43" s="17" t="n">
@@ -36637,7 +36637,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Подписки: сайт Shopify, домен, GPT, Claude, музыка</t>
+          <t xml:space="preserve">        Подписки и сервисы: сайт, домен, музыка, программы</t>
         </is>
       </c>
       <c r="B53" s="17" t="n">
@@ -49064,7 +49064,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">        События и маркеты: грузчики, диджей, расходники</t>
+          <t xml:space="preserve">        События и маркеты: грузчики, музыка, расходники</t>
         </is>
       </c>
       <c r="B43" s="17" t="n">
@@ -50634,7 +50634,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Подписки: сайт Shopify, домен, GPT, Claude, музыка</t>
+          <t xml:space="preserve">        Подписки и сервисы: сайт, домен, музыка, программы</t>
         </is>
       </c>
       <c r="B53" s="17" t="n">
@@ -57221,7 +57221,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Подписки: сайт Shopify, домен, GPT, Claude, музыка</t>
+          <t>Подписки и сервисы: сайт, домен, музыка, программы</t>
         </is>
       </c>
       <c r="B45" s="22" t="n">
@@ -57271,7 +57271,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>События и маркеты: грузчики, диджей, расходники, со ступени B</t>
+          <t>События и маркеты: грузчики, музыка, расходники, со ступени B</t>
         </is>
       </c>
       <c r="B50" s="22" t="n">

</xml_diff>

<commit_message>
fix: deal fee named as placement fee 5%, screens 04 and 07 rewritten
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model-v7/maison-financial-model.xlsx
+++ b/model-v7/maison-financial-model.xlsx
@@ -11783,7 +11783,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Подготовка и оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ за модель, презентацию и переговоры</t>
+          <t xml:space="preserve">    Оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ вознаграждение за привлечение инвестиции (5% от суммы, по рынку 3-7%)</t>
         </is>
       </c>
       <c r="B73" s="17" t="n">
@@ -25780,7 +25780,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Подготовка и оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ за модель, презентацию и переговоры</t>
+          <t xml:space="preserve">    Оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ вознаграждение за привлечение инвестиции (5% от суммы, по рынку 3-7%)</t>
         </is>
       </c>
       <c r="B73" s="17" t="n">
@@ -39777,7 +39777,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Подготовка и оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ за модель, презентацию и переговоры</t>
+          <t xml:space="preserve">    Оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ вознаграждение за привлечение инвестиции (5% от суммы, по рынку 3-7%)</t>
         </is>
       </c>
       <c r="B73" s="17" t="n">
@@ -53774,7 +53774,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Подготовка и оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ за модель, презентацию и переговоры</t>
+          <t xml:space="preserve">    Оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ вознаграждение за привлечение инвестиции (5% от суммы, по рынку 3-7%)</t>
         </is>
       </c>
       <c r="B73" s="17" t="n">
@@ -57370,7 +57370,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Подготовка и оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ за модель, презентацию и переговоры, 2026-12</t>
+          <t>Оформление сделки в день поступления денег: 2 000 $ нотариусу, 5 000 $ вознаграждение за привлечение инвестиции (5% от суммы, по рынку 3-7%), 2026-12</t>
         </is>
       </c>
       <c r="B61" s="22" t="n">

</xml_diff>